<commit_message>
Make the rating cell in Amanda's model calculate (shows HOLD)
The template had formatted Valuation!B54 as Text, so Amanda's IF formula was
stored as text. Her formula is unchanged; the cell now uses General format and
is a live formula, cached result HOLD.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Dx1iU5jAWd57T6rmzHCUf
</commit_message>
<xml_diff>
--- a/own-model/diageo-dcf-amanda-2026-10-16.xlsx
+++ b/own-model/diageo-dcf-amanda-2026-10-16.xlsx
@@ -618,7 +618,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -671,6 +671,7 @@
     <xf numFmtId="2" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2790,8 +2791,9 @@
       <c r="A54" t="s">
         <v>136</v>
       </c>
-      <c r="B54" s="18" t="s">
-        <v>151</v>
+      <c r="B54" s="42" t="str">
+        <f>IF(B53&gt;Inputs!B37,"BUY",IF(B53&lt;Inputs!B38,"SELL","HOLD"))</f>
+        <v>HOLD</v>
       </c>
       <c r="C54" s="36"/>
       <c r="D54" s="24"/>

</xml_diff>

<commit_message>
Rename the "Your answer" headings to "Value" and make the rating cell calculate in Amanda's Diageo model (#19)
* Rename the 'Your answer' headings to 'Value' in Amanda's Diageo model

Only the four column-heading labels change (WACC!B4, Valuation!B10, B39, B50).
Every formula and calculated value is untouched: 1,780.2p.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Dx1iU5jAWd57T6rmzHCUf

* Make the rating cell in Amanda's model calculate (shows HOLD)

The template had formatted Valuation!B54 as Text, so Amanda's IF formula was
stored as text. Her formula is unchanged; the cell now uses General format and
is a live formula, cached result HOLD.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Dx1iU5jAWd57T6rmzHCUf

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/own-model/diageo-dcf-amanda-2026-10-16.xlsx
+++ b/own-model/diageo-dcf-amanda-2026-10-16.xlsx
@@ -312,7 +312,7 @@
     <t>Step 3: WACC</t>
   </si>
   <si>
-    <t>Your answer</t>
+    <t>Value</t>
   </si>
   <si>
     <t>Market value of equity (market cap), USD m</t>
@@ -618,7 +618,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -671,6 +671,7 @@
     <xf numFmtId="2" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2790,8 +2791,9 @@
       <c r="A54" t="s">
         <v>136</v>
       </c>
-      <c r="B54" s="18" t="s">
-        <v>151</v>
+      <c r="B54" s="42" t="str">
+        <f>IF(B53&gt;Inputs!B37,"BUY",IF(B53&lt;Inputs!B38,"SELL","HOLD"))</f>
+        <v>HOLD</v>
       </c>
       <c r="C54" s="36"/>
       <c r="D54" s="24"/>

</xml_diff>